<commit_message>
this prompt consistently gets 95% precision but recall sucks, 68%
</commit_message>
<xml_diff>
--- a/output/df_small.xlsx
+++ b/output/df_small.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,6 +471,16 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>call_llm</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>lcs_score</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>alt_abbrev_response</t>
         </is>
       </c>
@@ -478,57 +488,60 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>HGNC:11540</t>
+          <t>HGNC:10201</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ENSG00000106290</t>
+          <t>ENSG00000283671, ENSG00000207047</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>GENE ID:6878</t>
+          <t>GENE ID:26798</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>TAF6</t>
+          <t>SNORD51</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>TAF(II)80</t>
+          <t>U51</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>TATA-box binding protein associated factor 6</t>
+          <t>small nucleolar RNA, C/D box 51</t>
         </is>
       </c>
       <c r="G2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: TAF(II)80
-    HGNC record ID: HGNC:11540
-    Primary gene symbol: TAF6
-    Official HGNC gene name: TATA-box binding protein associated factor 6
+    Alias gene symbol: U51
+    HGNC record ID: HGNC:10201
+    Primary gene symbol: SNORD51
+    Official HGNC gene name: small nucleolar RNA, C/D box 51
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
-    Note: If an alias symbol includes numerical characters not present in the primary gene symbol or gene name, 
-    it should not be classified as an Alternate Abbreviation no matter what criteria it meets.
     Classify the alias symbol as an Alternate Abbreviation if it meets at least one of these criteria:
-    1. If the letters in the alias symbol can be reasonably expanded to the official HGNC gene name, 
-    or to a phrase that is nearly identical in wording and meaning. 
+    1. If the alias symbol letters expand directly to the words present in the official HGNC gene name
+    or a nearly identical wording, while still uniquely identifying the same gene. 
     2. If the alias symbol differs from the primary gene symbol only by non-alphanumeric characters.
     3. If the alias symbol has the same alphanumeric order as the primary gene symbol but is truncated 
     through the removal of select characters. 
     4. Special case: Alias symbols for microRNA genes that have the "hsa" or "HSA" prefix are not
     Alternate Abbreviations while those without the "hsa" or "HSA" prefix are Alternate Abbreviations.
+    Notes for exclusion:
+    1. If an alias symbol includes numerical characters not present in the primary gene symbol or gene name,
+    it should not be classified as an Alternate Abbreviation no matter what criteria it meets.
+    2. Aliases derived from historical protein names, molecular weights, biochemical characterizations,
+    or gene family names should NOT be considered Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -541,26 +554,33 @@
     Rules:
     If the alias symbol is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the alias symbol is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias symbol is an alternate abbreviation, return:
+    "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "hgnc_id:"HGNC:11540"
-    "alias_symbol": "TAF(II)80",
-    "primary_gene_symbol": "TAF6",
-    "name": "TATA-box binding protein associated factor 6",
+    "hgnc_id":"HGNC:10201"
+    "alias_symbol": "U51",
+    "primary_gene_symbol": "SNORD51",
+    "name": "small nucleolar RNA, C/D box 51",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.2857142857142857</v>
+      </c>
+      <c r="K2" t="inlineStr">
         <is>
           <t>{
-"hgnc_id": "HGNC:11540",
-"alias_symbol": "TAF(II)80",
-"primary_gene_symbol": "TAF6",
-"name": "TATA-box binding protein associated factor 6",
-"alternate_abbreviation": "TRUE"
+"hgnc_id":"HGNC:10201",
+"alias_symbol": "U51",
+"primary_gene_symbol": "SNORD51",
+"name": "small nucleolar RNA, C/D box 51",
+"alternate_abbreviation": "FALSE"
 }</t>
         </is>
       </c>
@@ -568,57 +588,60 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HGNC:12474</t>
+          <t>HGNC:10346</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ENSG00000072401</t>
+          <t>ENSG00000165502</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>GENE ID:7321</t>
+          <t>GENE ID:6166</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>UBE2D1</t>
+          <t>RPL36AL</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>UBCH5</t>
+          <t>RPL36A</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>ubiquitin conjugating enzyme E2 D1</t>
+          <t>ribosomal protein L36a like</t>
         </is>
       </c>
       <c r="G3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: UBCH5
-    HGNC record ID: HGNC:12474
-    Primary gene symbol: UBE2D1
-    Official HGNC gene name: ubiquitin conjugating enzyme E2 D1
+    Alias gene symbol: RPL36A
+    HGNC record ID: HGNC:10346
+    Primary gene symbol: RPL36AL
+    Official HGNC gene name: ribosomal protein L36a like
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
-    Note: If an alias symbol includes numerical characters not present in the primary gene symbol or gene name, 
-    it should not be classified as an Alternate Abbreviation no matter what criteria it meets.
     Classify the alias symbol as an Alternate Abbreviation if it meets at least one of these criteria:
-    1. If the letters in the alias symbol can be reasonably expanded to the official HGNC gene name, 
-    or to a phrase that is nearly identical in wording and meaning. 
+    1. If the alias symbol letters expand directly to the words present in the official HGNC gene name
+    or a nearly identical wording, while still uniquely identifying the same gene. 
     2. If the alias symbol differs from the primary gene symbol only by non-alphanumeric characters.
     3. If the alias symbol has the same alphanumeric order as the primary gene symbol but is truncated 
     through the removal of select characters. 
     4. Special case: Alias symbols for microRNA genes that have the "hsa" or "HSA" prefix are not
     Alternate Abbreviations while those without the "hsa" or "HSA" prefix are Alternate Abbreviations.
+    Notes for exclusion:
+    1. If an alias symbol includes numerical characters not present in the primary gene symbol or gene name,
+    it should not be classified as an Alternate Abbreviation no matter what criteria it meets.
+    2. Aliases derived from historical protein names, molecular weights, biochemical characterizations,
+    or gene family names should NOT be considered Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -631,26 +654,33 @@
     Rules:
     If the alias symbol is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the alias symbol is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias symbol is an alternate abbreviation, return:
+    "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "hgnc_id:"HGNC:12474"
-    "alias_symbol": "UBCH5",
-    "primary_gene_symbol": "UBE2D1",
-    "name": "ubiquitin conjugating enzyme E2 D1",
+    "hgnc_id":"HGNC:10346"
+    "alias_symbol": "RPL36A",
+    "primary_gene_symbol": "RPL36AL",
+    "name": "ribosomal protein L36a like",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" t="b">
+        <v>1</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.8571428571428572</v>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t>{
-"hgnc_id": "HGNC:12474",
-"alias_symbol": "UBCH5",
-"primary_gene_symbol": "UBE2D1",
-"name": "ubiquitin conjugating enzyme E2 D1",
-"alternate_abbreviation": "TRUE"
+"hgnc_id": "HGNC:10346",
+"alias_symbol": "RPL36A",
+"primary_gene_symbol": "RPL36AL",
+"name": "ribosomal protein L36a like",
+"alternate_abbreviation": "FALSE"
 }</t>
         </is>
       </c>
@@ -658,57 +688,60 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HGNC:16046</t>
+          <t>HGNC:12195</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ENSG00000115446</t>
+          <t>ENSG00000226660, ENSG00000282568</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>GENE ID:25972</t>
+          <t>GENE ID:28620</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>UNC50</t>
+          <t>TRBV2</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>UNCL</t>
+          <t>TCRBV22S1A2N1T</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>unc-50 inner nuclear membrane RNA binding protein</t>
+          <t>T cell receptor beta variable 2</t>
         </is>
       </c>
       <c r="G4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: UNCL
-    HGNC record ID: HGNC:16046
-    Primary gene symbol: UNC50
-    Official HGNC gene name: unc-50 inner nuclear membrane RNA binding protein
+    Alias gene symbol: TCRBV22S1A2N1T
+    HGNC record ID: HGNC:12195
+    Primary gene symbol: TRBV2
+    Official HGNC gene name: T cell receptor beta variable 2
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
-    Note: If an alias symbol includes numerical characters not present in the primary gene symbol or gene name, 
-    it should not be classified as an Alternate Abbreviation no matter what criteria it meets.
     Classify the alias symbol as an Alternate Abbreviation if it meets at least one of these criteria:
-    1. If the letters in the alias symbol can be reasonably expanded to the official HGNC gene name, 
-    or to a phrase that is nearly identical in wording and meaning. 
+    1. If the alias symbol letters expand directly to the words present in the official HGNC gene name
+    or a nearly identical wording, while still uniquely identifying the same gene. 
     2. If the alias symbol differs from the primary gene symbol only by non-alphanumeric characters.
     3. If the alias symbol has the same alphanumeric order as the primary gene symbol but is truncated 
     through the removal of select characters. 
     4. Special case: Alias symbols for microRNA genes that have the "hsa" or "HSA" prefix are not
     Alternate Abbreviations while those without the "hsa" or "HSA" prefix are Alternate Abbreviations.
+    Notes for exclusion:
+    1. If an alias symbol includes numerical characters not present in the primary gene symbol or gene name,
+    it should not be classified as an Alternate Abbreviation no matter what criteria it meets.
+    2. Aliases derived from historical protein names, molecular weights, biochemical characterizations,
+    or gene family names should NOT be considered Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -721,26 +754,33 @@
     Rules:
     If the alias symbol is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the alias symbol is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias symbol is an alternate abbreviation, return:
+    "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "hgnc_id:"HGNC:16046"
-    "alias_symbol": "UNCL",
-    "primary_gene_symbol": "UNC50",
-    "name": "unc-50 inner nuclear membrane RNA binding protein",
+    "hgnc_id":"HGNC:12195"
+    "alias_symbol": "TCRBV22S1A2N1T",
+    "primary_gene_symbol": "TRBV2",
+    "name": "T cell receptor beta variable 2",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.3571428571428571</v>
+      </c>
+      <c r="K4" t="inlineStr">
         <is>
           <t>{
-"hgnc_id": "HGNC:16046",
-"alias_symbol": "UNCL",
-"primary_gene_symbol": "UNC50",
-"name": "unc-50 inner nuclear membrane RNA binding protein",
-"alternate_abbreviation": "TRUE"
+"hgnc_id":"HGNC:12195",
+"alias_symbol": "TCRBV22S1A2N1T",
+"primary_gene_symbol": "TRBV2",
+"name": "T cell receptor beta variable 2",
+"alternate_abbreviation": "FALSE"
 }</t>
         </is>
       </c>
@@ -748,57 +788,60 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>HGNC:19</t>
+          <t>HGNC:17005</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ENSG00000129673</t>
+          <t>ENSG00000136110</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>GENE ID:15</t>
+          <t>GENE ID:11061</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>AANAT</t>
+          <t>CNMD</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>SNAT</t>
+          <t>CHM-I</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>aralkylamine N-acetyltransferase</t>
+          <t>chondromodulin</t>
         </is>
       </c>
       <c r="G5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: SNAT
-    HGNC record ID: HGNC:19
-    Primary gene symbol: AANAT
-    Official HGNC gene name: aralkylamine N-acetyltransferase
+    Alias gene symbol: CHM-I
+    HGNC record ID: HGNC:17005
+    Primary gene symbol: CNMD
+    Official HGNC gene name: chondromodulin
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
-    Note: If an alias symbol includes numerical characters not present in the primary gene symbol or gene name, 
-    it should not be classified as an Alternate Abbreviation no matter what criteria it meets.
     Classify the alias symbol as an Alternate Abbreviation if it meets at least one of these criteria:
-    1. If the letters in the alias symbol can be reasonably expanded to the official HGNC gene name, 
-    or to a phrase that is nearly identical in wording and meaning. 
+    1. If the alias symbol letters expand directly to the words present in the official HGNC gene name
+    or a nearly identical wording, while still uniquely identifying the same gene. 
     2. If the alias symbol differs from the primary gene symbol only by non-alphanumeric characters.
     3. If the alias symbol has the same alphanumeric order as the primary gene symbol but is truncated 
     through the removal of select characters. 
     4. Special case: Alias symbols for microRNA genes that have the "hsa" or "HSA" prefix are not
     Alternate Abbreviations while those without the "hsa" or "HSA" prefix are Alternate Abbreviations.
+    Notes for exclusion:
+    1. If an alias symbol includes numerical characters not present in the primary gene symbol or gene name,
+    it should not be classified as an Alternate Abbreviation no matter what criteria it meets.
+    2. Aliases derived from historical protein names, molecular weights, biochemical characterizations,
+    or gene family names should NOT be considered Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -811,25 +854,32 @@
     Rules:
     If the alias symbol is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the alias symbol is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias symbol is an alternate abbreviation, return:
+    "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "hgnc_id:"HGNC:19"
-    "alias_symbol": "SNAT",
-    "primary_gene_symbol": "AANAT",
-    "name": "aralkylamine N-acetyltransferase",
+    "hgnc_id":"HGNC:17005"
+    "alias_symbol": "CHM-I",
+    "primary_gene_symbol": "CNMD",
+    "name": "chondromodulin",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" t="b">
+        <v>1</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>{
-"hgnc_id": "HGNC:19",
-"alias_symbol": "SNAT",
-"primary_gene_symbol": "AANAT",
-"name": "aralkylamine N-acetyltransferase",
+"hgnc_id":"HGNC:17005",
+"alias_symbol": "CHM-I",
+"primary_gene_symbol": "CNMD",
+"name": "chondromodulin",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -838,57 +888,60 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>HGNC:20182</t>
+          <t>HGNC:17780</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ENSG00000029364</t>
+          <t>ENSG00000169067</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>GENE ID:55334</t>
+          <t>GENE ID:345651</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>SLC39A9</t>
+          <t>ACTBL2</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ZIP-9</t>
+          <t>ACT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>solute carrier family 39 member 9</t>
+          <t>actin beta like 2</t>
         </is>
       </c>
       <c r="G6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: ZIP-9
-    HGNC record ID: HGNC:20182
-    Primary gene symbol: SLC39A9
-    Official HGNC gene name: solute carrier family 39 member 9
+    Alias gene symbol: ACT
+    HGNC record ID: HGNC:17780
+    Primary gene symbol: ACTBL2
+    Official HGNC gene name: actin beta like 2
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
-    Note: If an alias symbol includes numerical characters not present in the primary gene symbol or gene name, 
-    it should not be classified as an Alternate Abbreviation no matter what criteria it meets.
     Classify the alias symbol as an Alternate Abbreviation if it meets at least one of these criteria:
-    1. If the letters in the alias symbol can be reasonably expanded to the official HGNC gene name, 
-    or to a phrase that is nearly identical in wording and meaning. 
+    1. If the alias symbol letters expand directly to the words present in the official HGNC gene name
+    or a nearly identical wording, while still uniquely identifying the same gene. 
     2. If the alias symbol differs from the primary gene symbol only by non-alphanumeric characters.
     3. If the alias symbol has the same alphanumeric order as the primary gene symbol but is truncated 
     through the removal of select characters. 
     4. Special case: Alias symbols for microRNA genes that have the "hsa" or "HSA" prefix are not
     Alternate Abbreviations while those without the "hsa" or "HSA" prefix are Alternate Abbreviations.
+    Notes for exclusion:
+    1. If an alias symbol includes numerical characters not present in the primary gene symbol or gene name,
+    it should not be classified as an Alternate Abbreviation no matter what criteria it meets.
+    2. Aliases derived from historical protein names, molecular weights, biochemical characterizations,
+    or gene family names should NOT be considered Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -901,25 +954,32 @@
     Rules:
     If the alias symbol is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the alias symbol is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias symbol is an alternate abbreviation, return:
+    "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "hgnc_id:"HGNC:20182"
-    "alias_symbol": "ZIP-9",
-    "primary_gene_symbol": "SLC39A9",
-    "name": "solute carrier family 39 member 9",
+    "hgnc_id":"HGNC:17780"
+    "alias_symbol": "ACT",
+    "primary_gene_symbol": "ACTBL2",
+    "name": "actin beta like 2",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I6" t="b">
+        <v>1</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K6" t="inlineStr">
         <is>
           <t>{
-"hgnc_id": "HGNC:20182",
-"alias_symbol": "ZIP-9",
-"primary_gene_symbol": "SLC39A9",
-"name": "solute carrier family 39 member 9",
+"hgnc_id":"HGNC:17780",
+"alias_symbol": "ACT",
+"primary_gene_symbol": "ACTBL2",
+"name": "actin beta like 2",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -928,57 +988,60 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>HGNC:27882</t>
+          <t>HGNC:18949</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ENSG00000247151</t>
+          <t>ENSG00000227840</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>GENE ID:338739</t>
+          <t>GENE ID:337981</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>CSTF3-DT</t>
+          <t>KRTAP8-3P</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CSTF3-AS1</t>
+          <t>KRTAP8P2</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>CSTF3 divergent transcript</t>
+          <t>keratin associated protein 8-3, pseudogene</t>
         </is>
       </c>
       <c r="G7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: CSTF3-AS1
-    HGNC record ID: HGNC:27882
-    Primary gene symbol: CSTF3-DT
-    Official HGNC gene name: CSTF3 divergent transcript
+    Alias gene symbol: KRTAP8P2
+    HGNC record ID: HGNC:18949
+    Primary gene symbol: KRTAP8-3P
+    Official HGNC gene name: keratin associated protein 8-3, pseudogene
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
-    Note: If an alias symbol includes numerical characters not present in the primary gene symbol or gene name, 
-    it should not be classified as an Alternate Abbreviation no matter what criteria it meets.
     Classify the alias symbol as an Alternate Abbreviation if it meets at least one of these criteria:
-    1. If the letters in the alias symbol can be reasonably expanded to the official HGNC gene name, 
-    or to a phrase that is nearly identical in wording and meaning. 
+    1. If the alias symbol letters expand directly to the words present in the official HGNC gene name
+    or a nearly identical wording, while still uniquely identifying the same gene. 
     2. If the alias symbol differs from the primary gene symbol only by non-alphanumeric characters.
     3. If the alias symbol has the same alphanumeric order as the primary gene symbol but is truncated 
     through the removal of select characters. 
     4. Special case: Alias symbols for microRNA genes that have the "hsa" or "HSA" prefix are not
     Alternate Abbreviations while those without the "hsa" or "HSA" prefix are Alternate Abbreviations.
+    Notes for exclusion:
+    1. If an alias symbol includes numerical characters not present in the primary gene symbol or gene name,
+    it should not be classified as an Alternate Abbreviation no matter what criteria it meets.
+    2. Aliases derived from historical protein names, molecular weights, biochemical characterizations,
+    or gene family names should NOT be considered Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -991,26 +1054,33 @@
     Rules:
     If the alias symbol is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the alias symbol is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias symbol is an alternate abbreviation, return:
+    "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "hgnc_id:"HGNC:27882"
-    "alias_symbol": "CSTF3-AS1",
-    "primary_gene_symbol": "CSTF3-DT",
-    "name": "CSTF3 divergent transcript",
+    "hgnc_id":"HGNC:18949"
+    "alias_symbol": "KRTAP8P2",
+    "primary_gene_symbol": "KRTAP8-3P",
+    "name": "keratin associated protein 8-3, pseudogene",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" t="b">
+        <v>1</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="K7" t="inlineStr">
         <is>
           <t>{
-"hgnc_id": "HGNC:27882",
-"alias_symbol": "CSTF3-AS1",
-"primary_gene_symbol": "CSTF3-DT",
-"name": "CSTF3 divergent transcript",
-"alternate_abbreviation": "FALSE"
+    "hgnc_id": "HGNC:18949",
+    "alias_symbol": "KRTAP8P2",
+    "primary_gene_symbol": "KRTAP8-3P",
+    "name": "keratin associated protein 8-3, pseudogene",
+    "alternate_abbreviation": "TRUE"
 }</t>
         </is>
       </c>
@@ -1018,57 +1088,60 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HGNC:34981</t>
+          <t>HGNC:24086</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>set()</t>
+          <t>ENSG00000148584</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>GENE ID:100189412</t>
+          <t>GENE ID:29974</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>TRD-GTC2-1</t>
+          <t>A1CF</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>TRNAD18</t>
+          <t>ACF64</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>tRNA-Asp (anticodon GTC) 2-1</t>
+          <t>APOBEC1 complementation factor</t>
         </is>
       </c>
       <c r="G8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: TRNAD18
-    HGNC record ID: HGNC:34981
-    Primary gene symbol: TRD-GTC2-1
-    Official HGNC gene name: tRNA-Asp (anticodon GTC) 2-1
+    Alias gene symbol: ACF64
+    HGNC record ID: HGNC:24086
+    Primary gene symbol: A1CF
+    Official HGNC gene name: APOBEC1 complementation factor
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
-    Note: If an alias symbol includes numerical characters not present in the primary gene symbol or gene name, 
-    it should not be classified as an Alternate Abbreviation no matter what criteria it meets.
     Classify the alias symbol as an Alternate Abbreviation if it meets at least one of these criteria:
-    1. If the letters in the alias symbol can be reasonably expanded to the official HGNC gene name, 
-    or to a phrase that is nearly identical in wording and meaning. 
+    1. If the alias symbol letters expand directly to the words present in the official HGNC gene name
+    or a nearly identical wording, while still uniquely identifying the same gene. 
     2. If the alias symbol differs from the primary gene symbol only by non-alphanumeric characters.
     3. If the alias symbol has the same alphanumeric order as the primary gene symbol but is truncated 
     through the removal of select characters. 
     4. Special case: Alias symbols for microRNA genes that have the "hsa" or "HSA" prefix are not
     Alternate Abbreviations while those without the "hsa" or "HSA" prefix are Alternate Abbreviations.
+    Notes for exclusion:
+    1. If an alias symbol includes numerical characters not present in the primary gene symbol or gene name,
+    it should not be classified as an Alternate Abbreviation no matter what criteria it meets.
+    2. Aliases derived from historical protein names, molecular weights, biochemical characterizations,
+    or gene family names should NOT be considered Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -1081,25 +1154,32 @@
     Rules:
     If the alias symbol is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the alias symbol is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias symbol is an alternate abbreviation, return:
+    "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "hgnc_id:"HGNC:34981"
-    "alias_symbol": "TRNAD18",
-    "primary_gene_symbol": "TRD-GTC2-1",
-    "name": "tRNA-Asp (anticodon GTC) 2-1",
+    "hgnc_id":"HGNC:24086"
+    "alias_symbol": "ACF64",
+    "primary_gene_symbol": "A1CF",
+    "name": "APOBEC1 complementation factor",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I8" t="b">
+        <v>1</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="K8" t="inlineStr">
         <is>
           <t>{
-"hgnc_id": "HGNC:34981",
-"alias_symbol": "TRNAD18",
-"primary_gene_symbol": "TRD-GTC2-1",
-"name": "tRNA-Asp (anticodon GTC) 2-1",
+"hgnc_id":"HGNC:24086",
+"alias_symbol": "ACF64",
+"primary_gene_symbol": "A1CF",
+"name": "APOBEC1 complementation factor",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -1108,57 +1188,60 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>HGNC:38866</t>
+          <t>HGNC:318</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ENSG00000250709</t>
+          <t>ENSG00000038002</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>GENE ID:100526761</t>
+          <t>GENE ID:175</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>CCDC169-SOHLH2</t>
+          <t>AGA</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>C13orf38-SOHLH2</t>
+          <t>ASRG</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>CCDC169-SOHLH2 readthrough</t>
+          <t>aspartylglucosaminidase</t>
         </is>
       </c>
       <c r="G9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: C13orf38-SOHLH2
-    HGNC record ID: HGNC:38866
-    Primary gene symbol: CCDC169-SOHLH2
-    Official HGNC gene name: CCDC169-SOHLH2 readthrough
+    Alias gene symbol: ASRG
+    HGNC record ID: HGNC:318
+    Primary gene symbol: AGA
+    Official HGNC gene name: aspartylglucosaminidase
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
-    Note: If an alias symbol includes numerical characters not present in the primary gene symbol or gene name, 
-    it should not be classified as an Alternate Abbreviation no matter what criteria it meets.
     Classify the alias symbol as an Alternate Abbreviation if it meets at least one of these criteria:
-    1. If the letters in the alias symbol can be reasonably expanded to the official HGNC gene name, 
-    or to a phrase that is nearly identical in wording and meaning. 
+    1. If the alias symbol letters expand directly to the words present in the official HGNC gene name
+    or a nearly identical wording, while still uniquely identifying the same gene. 
     2. If the alias symbol differs from the primary gene symbol only by non-alphanumeric characters.
     3. If the alias symbol has the same alphanumeric order as the primary gene symbol but is truncated 
     through the removal of select characters. 
     4. Special case: Alias symbols for microRNA genes that have the "hsa" or "HSA" prefix are not
     Alternate Abbreviations while those without the "hsa" or "HSA" prefix are Alternate Abbreviations.
+    Notes for exclusion:
+    1. If an alias symbol includes numerical characters not present in the primary gene symbol or gene name,
+    it should not be classified as an Alternate Abbreviation no matter what criteria it meets.
+    2. Aliases derived from historical protein names, molecular weights, biochemical characterizations,
+    or gene family names should NOT be considered Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -1171,25 +1254,32 @@
     Rules:
     If the alias symbol is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the alias symbol is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias symbol is an alternate abbreviation, return:
+    "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "hgnc_id:"HGNC:38866"
-    "alias_symbol": "C13orf38-SOHLH2",
-    "primary_gene_symbol": "CCDC169-SOHLH2",
-    "name": "CCDC169-SOHLH2 readthrough",
+    "hgnc_id":"HGNC:318"
+    "alias_symbol": "ASRG",
+    "primary_gene_symbol": "AGA",
+    "name": "aspartylglucosaminidase",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I9" t="b">
+        <v>1</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K9" t="inlineStr">
         <is>
           <t>{
-"hgnc_id": "HGNC:38866",
-"alias_symbol": "C13orf38-SOHLH2",
-"primary_gene_symbol": "CCDC169-SOHLH2",
-"name": "CCDC169-SOHLH2 readthrough",
+"hgnc_id":"HGNC:318",
+"alias_symbol": "ASRG",
+"primary_gene_symbol": "AGA",
+"name": "aspartylglucosaminidase",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -1198,57 +1288,60 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>HGNC:5880</t>
+          <t>HGNC:32419</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ENSG00000211648</t>
+          <t>ENSG00000183054</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>GENE ID:28822</t>
+          <t>GENE ID:729540</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>IGLV1-47</t>
+          <t>RGPD6</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>V1-17</t>
+          <t>RanBP2L2</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>immunoglobulin lambda variable 1-47</t>
+          <t>RANBP2 like and GRIP domain containing 6</t>
         </is>
       </c>
       <c r="G10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: V1-17
-    HGNC record ID: HGNC:5880
-    Primary gene symbol: IGLV1-47
-    Official HGNC gene name: immunoglobulin lambda variable 1-47
+    Alias gene symbol: RanBP2L2
+    HGNC record ID: HGNC:32419
+    Primary gene symbol: RGPD6
+    Official HGNC gene name: RANBP2 like and GRIP domain containing 6
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
-    Note: If an alias symbol includes numerical characters not present in the primary gene symbol or gene name, 
-    it should not be classified as an Alternate Abbreviation no matter what criteria it meets.
     Classify the alias symbol as an Alternate Abbreviation if it meets at least one of these criteria:
-    1. If the letters in the alias symbol can be reasonably expanded to the official HGNC gene name, 
-    or to a phrase that is nearly identical in wording and meaning. 
+    1. If the alias symbol letters expand directly to the words present in the official HGNC gene name
+    or a nearly identical wording, while still uniquely identifying the same gene. 
     2. If the alias symbol differs from the primary gene symbol only by non-alphanumeric characters.
     3. If the alias symbol has the same alphanumeric order as the primary gene symbol but is truncated 
     through the removal of select characters. 
     4. Special case: Alias symbols for microRNA genes that have the "hsa" or "HSA" prefix are not
     Alternate Abbreviations while those without the "hsa" or "HSA" prefix are Alternate Abbreviations.
+    Notes for exclusion:
+    1. If an alias symbol includes numerical characters not present in the primary gene symbol or gene name,
+    it should not be classified as an Alternate Abbreviation no matter what criteria it meets.
+    2. Aliases derived from historical protein names, molecular weights, biochemical characterizations,
+    or gene family names should NOT be considered Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -1261,25 +1354,32 @@
     Rules:
     If the alias symbol is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the alias symbol is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias symbol is an alternate abbreviation, return:
+    "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "hgnc_id:"HGNC:5880"
-    "alias_symbol": "V1-17",
-    "primary_gene_symbol": "IGLV1-47",
-    "name": "immunoglobulin lambda variable 1-47",
+    "hgnc_id":"HGNC:32419"
+    "alias_symbol": "RanBP2L2",
+    "primary_gene_symbol": "RGPD6",
+    "name": "RANBP2 like and GRIP domain containing 6",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I10" t="b">
+        <v>1</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K10" t="inlineStr">
         <is>
           <t>{
-"hgnc_id": "HGNC:5880",
-"alias_symbol": "V1-17",
-"primary_gene_symbol": "IGLV1-47",
-"name": "immunoglobulin lambda variable 1-47",
+"hgnc_id":"HGNC:32419",
+"alias_symbol": "RanBP2L2",
+"primary_gene_symbol": "RGPD6",
+"name": "RANBP2 like and GRIP domain containing 6",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -1288,57 +1388,60 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>HGNC:6345</t>
+          <t>HGNC:3308</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ENSG00000105610</t>
+          <t>ENSG00000139610</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>GENE ID:10661</t>
+          <t>GENE ID:1990</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>KLF1</t>
+          <t>CELA1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>EKLF/KLF1</t>
+          <t>ELA1</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>KLF transcription factor 1</t>
+          <t>chymotrypsin like elastase 1</t>
         </is>
       </c>
       <c r="G11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
           <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     Inputs:
-    Alias gene symbol: EKLF/KLF1
-    HGNC record ID: HGNC:6345
-    Primary gene symbol: KLF1
-    Official HGNC gene name: KLF transcription factor 1
+    Alias gene symbol: ELA1
+    HGNC record ID: HGNC:3308
+    Primary gene symbol: CELA1
+    Official HGNC gene name: chymotrypsin like elastase 1
     Task:
     Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
-    Note: If an alias symbol includes numerical characters not present in the primary gene symbol or gene name, 
-    it should not be classified as an Alternate Abbreviation no matter what criteria it meets.
     Classify the alias symbol as an Alternate Abbreviation if it meets at least one of these criteria:
-    1. If the letters in the alias symbol can be reasonably expanded to the official HGNC gene name, 
-    or to a phrase that is nearly identical in wording and meaning. 
+    1. If the alias symbol letters expand directly to the words present in the official HGNC gene name
+    or a nearly identical wording, while still uniquely identifying the same gene. 
     2. If the alias symbol differs from the primary gene symbol only by non-alphanumeric characters.
     3. If the alias symbol has the same alphanumeric order as the primary gene symbol but is truncated 
     through the removal of select characters. 
     4. Special case: Alias symbols for microRNA genes that have the "hsa" or "HSA" prefix are not
     Alternate Abbreviations while those without the "hsa" or "HSA" prefix are Alternate Abbreviations.
+    Notes for exclusion:
+    1. If an alias symbol includes numerical characters not present in the primary gene symbol or gene name,
+    it should not be classified as an Alternate Abbreviation no matter what criteria it meets.
+    2. Aliases derived from historical protein names, molecular weights, biochemical characterizations,
+    or gene family names should NOT be considered Alternate Abbreviations.
     Examples:
     1-
     Alias gene symbol: ACF65
@@ -1351,26 +1454,433 @@
     Rules:
     If the alias symbol is not an alternate abbreviation, return:
     "alternate_abbreviation": "FALSE"
-    If the alias symbol is an alternate abbreviation, set "alternate_abbreviation": "TRUE"
+    If the alias symbol is an alternate abbreviation, return:
+    "alternate_abbreviation": "TRUE"
     Output (Strict):
     Output only one JSON object. No markdown.
     {
-    "hgnc_id:"HGNC:6345"
-    "alias_symbol": "EKLF/KLF1",
-    "primary_gene_symbol": "KLF1",
-    "name": "KLF transcription factor 1",
+    "hgnc_id":"HGNC:3308"
+    "alias_symbol": "ELA1",
+    "primary_gene_symbol": "CELA1",
+    "name": "chymotrypsin like elastase 1",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I11" t="b">
+        <v>1</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K11" t="inlineStr">
         <is>
           <t>{
-"hgnc_id": "HGNC:6345",
-"alias_symbol": "EKLF/KLF1",
-"primary_gene_symbol": "KLF1",
-"name": "KLF transcription factor 1",
-"alternate_abbreviation": "TRUE"
+"hgnc_id":"HGNC:3308",
+"alias_symbol": "ELA1",
+"primary_gene_symbol": "CELA1",
+"name": "chymotrypsin like elastase 1",
+"alternate_abbreviation": "FALSE"
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>HGNC:42171</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ENSG00000232928</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>GENE ID:100133180</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>DDX3P1</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>DDX3YP1</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>DEAD-box helicase 3 pseudogene 1</t>
+        </is>
+      </c>
+      <c r="G12" t="b">
+        <v>1</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
+    Inputs:
+    Alias gene symbol: DDX3YP1
+    HGNC record ID: HGNC:42171
+    Primary gene symbol: DDX3P1
+    Official HGNC gene name: DEAD-box helicase 3 pseudogene 1
+    Task:
+    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
+    Classify the alias symbol as an Alternate Abbreviation if it meets at least one of these criteria:
+    1. If the alias symbol letters expand directly to the words present in the official HGNC gene name
+    or a nearly identical wording, while still uniquely identifying the same gene. 
+    2. If the alias symbol differs from the primary gene symbol only by non-alphanumeric characters.
+    3. If the alias symbol has the same alphanumeric order as the primary gene symbol but is truncated 
+    through the removal of select characters. 
+    4. Special case: Alias symbols for microRNA genes that have the "hsa" or "HSA" prefix are not
+    Alternate Abbreviations while those without the "hsa" or "HSA" prefix are Alternate Abbreviations.
+    Notes for exclusion:
+    1. If an alias symbol includes numerical characters not present in the primary gene symbol or gene name,
+    it should not be classified as an Alternate Abbreviation no matter what criteria it meets.
+    2. Aliases derived from historical protein names, molecular weights, biochemical characterizations,
+    or gene family names should NOT be considered Alternate Abbreviations.
+    Examples:
+    1-
+    Alias gene symbol: ACF65
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
+    2-
+    Alias gene symbol: ALPHA4GNT
+    Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
+    Primary gene symbol: A4GNT
+    Rules:
+    If the alias symbol is not an alternate abbreviation, return:
+    "alternate_abbreviation": "FALSE"
+    If the alias symbol is an alternate abbreviation, return:
+    "alternate_abbreviation": "TRUE"
+    Output (Strict):
+    Output only one JSON object. No markdown.
+    {
+    "hgnc_id":"HGNC:42171"
+    "alias_symbol": "DDX3YP1",
+    "primary_gene_symbol": "DDX3P1",
+    "name": "DEAD-box helicase 3 pseudogene 1",
+    "alternate_abbreviation": "TRUE or FALSE"
+    }</t>
+        </is>
+      </c>
+      <c r="I12" t="b">
+        <v>1</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.8571428571428572</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>{
+"hgnc_id":"HGNC:42171",
+"alias_symbol": "DDX3YP1",
+"primary_gene_symbol": "DDX3P1",
+"name": "DEAD-box helicase 3 pseudogene 1",
+"alternate_abbreviation": "FALSE"
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>HGNC:7505</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ENSG00000236675</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>GENE ID:4581</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>MTX1LP</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>psMTX</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>metaxin 1 like, pseudogene</t>
+        </is>
+      </c>
+      <c r="G13" t="b">
+        <v>1</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
+    Inputs:
+    Alias gene symbol: psMTX
+    HGNC record ID: HGNC:7505
+    Primary gene symbol: MTX1LP
+    Official HGNC gene name: metaxin 1 like, pseudogene
+    Task:
+    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
+    Classify the alias symbol as an Alternate Abbreviation if it meets at least one of these criteria:
+    1. If the alias symbol letters expand directly to the words present in the official HGNC gene name
+    or a nearly identical wording, while still uniquely identifying the same gene. 
+    2. If the alias symbol differs from the primary gene symbol only by non-alphanumeric characters.
+    3. If the alias symbol has the same alphanumeric order as the primary gene symbol but is truncated 
+    through the removal of select characters. 
+    4. Special case: Alias symbols for microRNA genes that have the "hsa" or "HSA" prefix are not
+    Alternate Abbreviations while those without the "hsa" or "HSA" prefix are Alternate Abbreviations.
+    Notes for exclusion:
+    1. If an alias symbol includes numerical characters not present in the primary gene symbol or gene name,
+    it should not be classified as an Alternate Abbreviation no matter what criteria it meets.
+    2. Aliases derived from historical protein names, molecular weights, biochemical characterizations,
+    or gene family names should NOT be considered Alternate Abbreviations.
+    Examples:
+    1-
+    Alias gene symbol: ACF65
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
+    2-
+    Alias gene symbol: ALPHA4GNT
+    Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
+    Primary gene symbol: A4GNT
+    Rules:
+    If the alias symbol is not an alternate abbreviation, return:
+    "alternate_abbreviation": "FALSE"
+    If the alias symbol is an alternate abbreviation, return:
+    "alternate_abbreviation": "TRUE"
+    Output (Strict):
+    Output only one JSON object. No markdown.
+    {
+    "hgnc_id":"HGNC:7505"
+    "alias_symbol": "psMTX",
+    "primary_gene_symbol": "MTX1LP",
+    "name": "metaxin 1 like, pseudogene",
+    "alternate_abbreviation": "TRUE or FALSE"
+    }</t>
+        </is>
+      </c>
+      <c r="I13" t="b">
+        <v>1</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>{
+    "hgnc_id": "HGNC:7505",
+    "alias_symbol": "psMTX",
+    "primary_gene_symbol": "MTX1LP",
+    "name": "metaxin 1 like, pseudogene",
+    "alternate_abbreviation": "FALSE"
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>HGNC:9366</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ENSG00000231887</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>GENE ID:5554</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>PRH1</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Pr1/Pr2</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>proline rich protein HaeIII subfamily 1</t>
+        </is>
+      </c>
+      <c r="G14" t="b">
+        <v>1</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
+    Inputs:
+    Alias gene symbol: Pr1/Pr2
+    HGNC record ID: HGNC:9366
+    Primary gene symbol: PRH1
+    Official HGNC gene name: proline rich protein HaeIII subfamily 1
+    Task:
+    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
+    Classify the alias symbol as an Alternate Abbreviation if it meets at least one of these criteria:
+    1. If the alias symbol letters expand directly to the words present in the official HGNC gene name
+    or a nearly identical wording, while still uniquely identifying the same gene. 
+    2. If the alias symbol differs from the primary gene symbol only by non-alphanumeric characters.
+    3. If the alias symbol has the same alphanumeric order as the primary gene symbol but is truncated 
+    through the removal of select characters. 
+    4. Special case: Alias symbols for microRNA genes that have the "hsa" or "HSA" prefix are not
+    Alternate Abbreviations while those without the "hsa" or "HSA" prefix are Alternate Abbreviations.
+    Notes for exclusion:
+    1. If an alias symbol includes numerical characters not present in the primary gene symbol or gene name,
+    it should not be classified as an Alternate Abbreviation no matter what criteria it meets.
+    2. Aliases derived from historical protein names, molecular weights, biochemical characterizations,
+    or gene family names should NOT be considered Alternate Abbreviations.
+    Examples:
+    1-
+    Alias gene symbol: ACF65
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
+    2-
+    Alias gene symbol: ALPHA4GNT
+    Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
+    Primary gene symbol: A4GNT
+    Rules:
+    If the alias symbol is not an alternate abbreviation, return:
+    "alternate_abbreviation": "FALSE"
+    If the alias symbol is an alternate abbreviation, return:
+    "alternate_abbreviation": "TRUE"
+    Output (Strict):
+    Output only one JSON object. No markdown.
+    {
+    "hgnc_id":"HGNC:9366"
+    "alias_symbol": "Pr1/Pr2",
+    "primary_gene_symbol": "PRH1",
+    "name": "proline rich protein HaeIII subfamily 1",
+    "alternate_abbreviation": "TRUE or FALSE"
+    }</t>
+        </is>
+      </c>
+      <c r="I14" t="b">
+        <v>1</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>{
+"hgnc_id":"HGNC:9366",
+"alias_symbol": "Pr1/Pr2",
+"primary_gene_symbol": "PRH1",
+"name": "proline rich protein HaeIII subfamily 1",
+"alternate_abbreviation": "FALSE"
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>HGNC:9969</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ENSG00000035928</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>GENE ID:5981</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>RFC1</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>RECC1</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>replication factor C subunit 1</t>
+        </is>
+      </c>
+      <c r="G15" t="b">
+        <v>1</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
+    Inputs:
+    Alias gene symbol: RECC1
+    HGNC record ID: HGNC:9969
+    Primary gene symbol: RFC1
+    Official HGNC gene name: replication factor C subunit 1
+    Task:
+    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
+    Classify the alias symbol as an Alternate Abbreviation if it meets at least one of these criteria:
+    1. If the alias symbol letters expand directly to the words present in the official HGNC gene name
+    or a nearly identical wording, while still uniquely identifying the same gene. 
+    2. If the alias symbol differs from the primary gene symbol only by non-alphanumeric characters.
+    3. If the alias symbol has the same alphanumeric order as the primary gene symbol but is truncated 
+    through the removal of select characters. 
+    4. Special case: Alias symbols for microRNA genes that have the "hsa" or "HSA" prefix are not
+    Alternate Abbreviations while those without the "hsa" or "HSA" prefix are Alternate Abbreviations.
+    Notes for exclusion:
+    1. If an alias symbol includes numerical characters not present in the primary gene symbol or gene name,
+    it should not be classified as an Alternate Abbreviation no matter what criteria it meets.
+    2. Aliases derived from historical protein names, molecular weights, biochemical characterizations,
+    or gene family names should NOT be considered Alternate Abbreviations.
+    Examples:
+    1-
+    Alias gene symbol: ACF65
+    Official HGNC gene name: APOBEC1 complementation factor
+    Primary gene symbol: A1CF
+    2-
+    Alias gene symbol: ALPHA4GNT
+    Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
+    Primary gene symbol: A4GNT
+    Rules:
+    If the alias symbol is not an alternate abbreviation, return:
+    "alternate_abbreviation": "FALSE"
+    If the alias symbol is an alternate abbreviation, return:
+    "alternate_abbreviation": "TRUE"
+    Output (Strict):
+    Output only one JSON object. No markdown.
+    {
+    "hgnc_id":"HGNC:9969"
+    "alias_symbol": "RECC1",
+    "primary_gene_symbol": "RFC1",
+    "name": "replication factor C subunit 1",
+    "alternate_abbreviation": "TRUE or FALSE"
+    }</t>
+        </is>
+      </c>
+      <c r="I15" t="b">
+        <v>1</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>{
+"hgnc_id":"HGNC:9969",
+"alias_symbol": "RECC1",
+"primary_gene_symbol": "RFC1",
+"name": "replication factor C subunit 1",
+"alternate_abbreviation": "FALSE"
 }</t>
         </is>
       </c>

</xml_diff>